<commit_message>
feat: validate demo client profile branding pipeline
</commit_message>
<xml_diff>
--- a/voucher_generator/LISTADO GENERAL - MODELO.xlsx
+++ b/voucher_generator/LISTADO GENERAL - MODELO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2bcce3142e000773/Escritorio/generadorDeVouchers/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ignac\Desktop\sharepoint_pipeline_app\voucher_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{057BF698-4BF1-4A3E-8887-0E579E22723B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF87C7B2-B11B-48D1-8062-53B8F3E74596}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724D405A-79FB-4FEF-9806-72E2199449F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" xr2:uid="{E92A6B87-369E-48A6-A293-58A76914B5E4}"/>
   </bookViews>
@@ -1423,39 +1423,81 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="12" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1479,48 +1521,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1914,76 +1914,76 @@
   <sheetData>
     <row r="1" spans="1:149" ht="12.75" customHeight="1">
       <c r="A1" s="38"/>
-      <c r="B1" s="143" t="s">
+      <c r="B1" s="164" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="144"/>
-      <c r="J1" s="144"/>
-      <c r="K1" s="144"/>
-      <c r="L1" s="144"/>
-      <c r="M1" s="144"/>
-      <c r="N1" s="144"/>
-      <c r="O1" s="144"/>
-      <c r="P1" s="144"/>
-      <c r="Q1" s="144"/>
-      <c r="R1" s="144"/>
-      <c r="S1" s="144"/>
-      <c r="T1" s="144"/>
-      <c r="U1" s="144"/>
-      <c r="V1" s="144"/>
-      <c r="W1" s="144"/>
-      <c r="X1" s="144"/>
-      <c r="Y1" s="144"/>
-      <c r="Z1" s="144"/>
-      <c r="AA1" s="144"/>
-      <c r="AB1" s="144"/>
-      <c r="AC1" s="144"/>
-      <c r="AD1" s="144"/>
-      <c r="AE1" s="144"/>
-      <c r="AF1" s="144"/>
-      <c r="AG1" s="144"/>
-      <c r="AH1" s="144"/>
-      <c r="AI1" s="144"/>
-      <c r="AJ1" s="144"/>
-      <c r="AK1" s="144"/>
-      <c r="AL1" s="144"/>
-      <c r="AM1" s="144"/>
-      <c r="AN1" s="144"/>
-      <c r="AO1" s="144"/>
-      <c r="AP1" s="144"/>
-      <c r="AQ1" s="144"/>
-      <c r="AR1" s="144"/>
-      <c r="AS1" s="144"/>
-      <c r="AT1" s="144"/>
-      <c r="AU1" s="144"/>
-      <c r="AV1" s="144"/>
-      <c r="AW1" s="144"/>
-      <c r="AX1" s="144"/>
-      <c r="AY1" s="144"/>
-      <c r="AZ1" s="144"/>
-      <c r="BA1" s="144"/>
-      <c r="BB1" s="144"/>
-      <c r="BC1" s="144"/>
-      <c r="BD1" s="144"/>
-      <c r="BE1" s="144"/>
-      <c r="BF1" s="144"/>
-      <c r="BG1" s="144"/>
-      <c r="BH1" s="144"/>
-      <c r="BI1" s="144"/>
-      <c r="BJ1" s="144"/>
-      <c r="BK1" s="144"/>
-      <c r="BL1" s="144"/>
-      <c r="BM1" s="144"/>
-      <c r="BN1" s="144"/>
-      <c r="BO1" s="144"/>
-      <c r="BP1" s="144"/>
-      <c r="BQ1" s="145"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
+      <c r="I1" s="157"/>
+      <c r="J1" s="157"/>
+      <c r="K1" s="157"/>
+      <c r="L1" s="157"/>
+      <c r="M1" s="157"/>
+      <c r="N1" s="157"/>
+      <c r="O1" s="157"/>
+      <c r="P1" s="157"/>
+      <c r="Q1" s="157"/>
+      <c r="R1" s="157"/>
+      <c r="S1" s="157"/>
+      <c r="T1" s="157"/>
+      <c r="U1" s="157"/>
+      <c r="V1" s="157"/>
+      <c r="W1" s="157"/>
+      <c r="X1" s="157"/>
+      <c r="Y1" s="157"/>
+      <c r="Z1" s="157"/>
+      <c r="AA1" s="157"/>
+      <c r="AB1" s="157"/>
+      <c r="AC1" s="157"/>
+      <c r="AD1" s="157"/>
+      <c r="AE1" s="157"/>
+      <c r="AF1" s="157"/>
+      <c r="AG1" s="157"/>
+      <c r="AH1" s="157"/>
+      <c r="AI1" s="157"/>
+      <c r="AJ1" s="157"/>
+      <c r="AK1" s="157"/>
+      <c r="AL1" s="157"/>
+      <c r="AM1" s="157"/>
+      <c r="AN1" s="157"/>
+      <c r="AO1" s="157"/>
+      <c r="AP1" s="157"/>
+      <c r="AQ1" s="157"/>
+      <c r="AR1" s="157"/>
+      <c r="AS1" s="157"/>
+      <c r="AT1" s="157"/>
+      <c r="AU1" s="157"/>
+      <c r="AV1" s="157"/>
+      <c r="AW1" s="157"/>
+      <c r="AX1" s="157"/>
+      <c r="AY1" s="157"/>
+      <c r="AZ1" s="157"/>
+      <c r="BA1" s="157"/>
+      <c r="BB1" s="157"/>
+      <c r="BC1" s="157"/>
+      <c r="BD1" s="157"/>
+      <c r="BE1" s="157"/>
+      <c r="BF1" s="157"/>
+      <c r="BG1" s="157"/>
+      <c r="BH1" s="157"/>
+      <c r="BI1" s="157"/>
+      <c r="BJ1" s="157"/>
+      <c r="BK1" s="157"/>
+      <c r="BL1" s="157"/>
+      <c r="BM1" s="157"/>
+      <c r="BN1" s="157"/>
+      <c r="BO1" s="157"/>
+      <c r="BP1" s="157"/>
+      <c r="BQ1" s="165"/>
       <c r="BR1" s="20"/>
       <c r="BS1" s="20"/>
       <c r="BT1" s="20"/>
@@ -2067,98 +2067,98 @@
     </row>
     <row r="2" spans="1:149" ht="15" customHeight="1">
       <c r="A2" s="39"/>
-      <c r="B2" s="157" t="s">
+      <c r="B2" s="171" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="161"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="175"/>
       <c r="E2" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="156" t="s">
+      <c r="G2" s="170" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="157"/>
-      <c r="N2" s="157"/>
-      <c r="O2" s="157"/>
-      <c r="P2" s="157"/>
-      <c r="Q2" s="157"/>
-      <c r="R2" s="157"/>
-      <c r="S2" s="157"/>
-      <c r="T2" s="157"/>
-      <c r="U2" s="161"/>
-      <c r="V2" s="153" t="s">
+      <c r="H2" s="171"/>
+      <c r="I2" s="171"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="171"/>
+      <c r="L2" s="171"/>
+      <c r="M2" s="171"/>
+      <c r="N2" s="171"/>
+      <c r="O2" s="171"/>
+      <c r="P2" s="171"/>
+      <c r="Q2" s="171"/>
+      <c r="R2" s="171"/>
+      <c r="S2" s="171"/>
+      <c r="T2" s="171"/>
+      <c r="U2" s="175"/>
+      <c r="V2" s="158" t="s">
         <v>5</v>
       </c>
-      <c r="W2" s="153"/>
-      <c r="X2" s="153"/>
-      <c r="Y2" s="153"/>
-      <c r="Z2" s="153"/>
-      <c r="AA2" s="153"/>
-      <c r="AB2" s="153"/>
-      <c r="AC2" s="152" t="s">
+      <c r="W2" s="158"/>
+      <c r="X2" s="158"/>
+      <c r="Y2" s="158"/>
+      <c r="Z2" s="158"/>
+      <c r="AA2" s="158"/>
+      <c r="AB2" s="158"/>
+      <c r="AC2" s="159" t="s">
         <v>6</v>
       </c>
-      <c r="AD2" s="153"/>
-      <c r="AE2" s="153"/>
-      <c r="AF2" s="153"/>
-      <c r="AG2" s="153"/>
-      <c r="AH2" s="153"/>
-      <c r="AI2" s="162"/>
-      <c r="AJ2" s="144" t="s">
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="158"/>
+      <c r="AF2" s="158"/>
+      <c r="AG2" s="158"/>
+      <c r="AH2" s="158"/>
+      <c r="AI2" s="160"/>
+      <c r="AJ2" s="157" t="s">
         <v>7</v>
       </c>
-      <c r="AK2" s="144"/>
-      <c r="AL2" s="144"/>
-      <c r="AM2" s="144"/>
-      <c r="AN2" s="144"/>
-      <c r="AO2" s="144"/>
-      <c r="AP2" s="144"/>
-      <c r="AQ2" s="152" t="s">
+      <c r="AK2" s="157"/>
+      <c r="AL2" s="157"/>
+      <c r="AM2" s="157"/>
+      <c r="AN2" s="157"/>
+      <c r="AO2" s="157"/>
+      <c r="AP2" s="157"/>
+      <c r="AQ2" s="159" t="s">
         <v>8</v>
       </c>
-      <c r="AR2" s="153"/>
-      <c r="AS2" s="153"/>
-      <c r="AT2" s="153"/>
-      <c r="AU2" s="153"/>
-      <c r="AV2" s="153"/>
-      <c r="AW2" s="153"/>
-      <c r="AX2" s="152" t="s">
+      <c r="AR2" s="158"/>
+      <c r="AS2" s="158"/>
+      <c r="AT2" s="158"/>
+      <c r="AU2" s="158"/>
+      <c r="AV2" s="158"/>
+      <c r="AW2" s="158"/>
+      <c r="AX2" s="159" t="s">
         <v>9</v>
       </c>
-      <c r="AY2" s="153"/>
-      <c r="AZ2" s="153"/>
-      <c r="BA2" s="153"/>
-      <c r="BB2" s="153"/>
-      <c r="BC2" s="153"/>
-      <c r="BD2" s="153"/>
-      <c r="BE2" s="154" t="s">
+      <c r="AY2" s="158"/>
+      <c r="AZ2" s="158"/>
+      <c r="BA2" s="158"/>
+      <c r="BB2" s="158"/>
+      <c r="BC2" s="158"/>
+      <c r="BD2" s="158"/>
+      <c r="BE2" s="168" t="s">
         <v>2</v>
       </c>
-      <c r="BF2" s="155"/>
-      <c r="BG2" s="156" t="s">
+      <c r="BF2" s="169"/>
+      <c r="BG2" s="170" t="s">
         <v>10</v>
       </c>
-      <c r="BH2" s="157"/>
-      <c r="BI2" s="158" t="s">
+      <c r="BH2" s="171"/>
+      <c r="BI2" s="172" t="s">
         <v>11</v>
       </c>
-      <c r="BJ2" s="159"/>
-      <c r="BK2" s="159"/>
-      <c r="BL2" s="159"/>
-      <c r="BM2" s="159"/>
-      <c r="BN2" s="159"/>
-      <c r="BO2" s="159"/>
-      <c r="BP2" s="159"/>
-      <c r="BQ2" s="160"/>
+      <c r="BJ2" s="173"/>
+      <c r="BK2" s="173"/>
+      <c r="BL2" s="173"/>
+      <c r="BM2" s="173"/>
+      <c r="BN2" s="173"/>
+      <c r="BO2" s="173"/>
+      <c r="BP2" s="173"/>
+      <c r="BQ2" s="174"/>
       <c r="BR2" s="20"/>
       <c r="BS2" s="20"/>
       <c r="BT2" s="20"/>
@@ -2533,13 +2533,13 @@
       <c r="A4" s="68">
         <v>1</v>
       </c>
-      <c r="B4" s="148" t="s">
+      <c r="B4" s="152" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="146" t="s">
+      <c r="C4" s="155" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="146" t="s">
+      <c r="D4" s="155" t="s">
         <v>61</v>
       </c>
       <c r="E4" s="68"/>
@@ -2619,7 +2619,7 @@
       <c r="AI4" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ4" s="150">
+      <c r="AJ4" s="166">
         <v>1</v>
       </c>
       <c r="AK4" s="141" t="s">
@@ -2628,16 +2628,16 @@
       <c r="AL4" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM4" s="150" t="s">
+      <c r="AM4" s="166" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="151">
+      <c r="AN4" s="167">
         <v>45709</v>
       </c>
-      <c r="AO4" s="151">
+      <c r="AO4" s="167">
         <v>45715</v>
       </c>
-      <c r="AP4" s="150">
+      <c r="AP4" s="166">
         <v>6</v>
       </c>
       <c r="AQ4" s="69" t="s">
@@ -2798,9 +2798,9 @@
       <c r="A5" s="81">
         <v>2</v>
       </c>
-      <c r="B5" s="149"/>
-      <c r="C5" s="147"/>
-      <c r="D5" s="147"/>
+      <c r="B5" s="153"/>
+      <c r="C5" s="156"/>
+      <c r="D5" s="156"/>
       <c r="E5" s="81"/>
       <c r="F5" s="82" t="s">
         <v>62</v>
@@ -2870,17 +2870,17 @@
       <c r="AI5" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ5" s="149"/>
+      <c r="AJ5" s="153"/>
       <c r="AK5" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL5" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM5" s="149"/>
-      <c r="AN5" s="149"/>
-      <c r="AO5" s="149"/>
-      <c r="AP5" s="149"/>
+      <c r="AM5" s="153"/>
+      <c r="AN5" s="153"/>
+      <c r="AO5" s="153"/>
+      <c r="AP5" s="153"/>
       <c r="AQ5" s="82" t="s">
         <v>75</v>
       </c>
@@ -3039,13 +3039,13 @@
       <c r="A6" s="110">
         <v>1</v>
       </c>
-      <c r="B6" s="170" t="s">
+      <c r="B6" s="151" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="171" t="s">
+      <c r="C6" s="154" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="171" t="s">
+      <c r="D6" s="154" t="s">
         <v>61</v>
       </c>
       <c r="E6" s="110"/>
@@ -3131,7 +3131,7 @@
       <c r="AI6" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ6" s="170">
+      <c r="AJ6" s="151">
         <v>1</v>
       </c>
       <c r="AK6" s="141" t="s">
@@ -3140,16 +3140,16 @@
       <c r="AL6" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM6" s="170" t="s">
+      <c r="AM6" s="151" t="s">
         <v>74</v>
       </c>
-      <c r="AN6" s="167">
+      <c r="AN6" s="161">
         <v>46104</v>
       </c>
-      <c r="AO6" s="167">
+      <c r="AO6" s="161">
         <v>46110</v>
       </c>
-      <c r="AP6" s="170">
+      <c r="AP6" s="151">
         <v>6</v>
       </c>
       <c r="AQ6" s="111" t="s">
@@ -3304,9 +3304,9 @@
       <c r="A7" s="125">
         <v>2</v>
       </c>
-      <c r="B7" s="148"/>
-      <c r="C7" s="146"/>
-      <c r="D7" s="146"/>
+      <c r="B7" s="152"/>
+      <c r="C7" s="155"/>
+      <c r="D7" s="155"/>
       <c r="E7" s="125"/>
       <c r="F7" s="111" t="s">
         <v>62</v>
@@ -3386,17 +3386,17 @@
       <c r="AI7" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ7" s="148"/>
+      <c r="AJ7" s="152"/>
       <c r="AK7" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL7" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM7" s="148"/>
-      <c r="AN7" s="168"/>
-      <c r="AO7" s="168"/>
-      <c r="AP7" s="148"/>
+      <c r="AM7" s="152"/>
+      <c r="AN7" s="162"/>
+      <c r="AO7" s="162"/>
+      <c r="AP7" s="152"/>
       <c r="AQ7" s="111" t="s">
         <v>92</v>
       </c>
@@ -3549,9 +3549,9 @@
       <c r="A8" s="81">
         <v>3</v>
       </c>
-      <c r="B8" s="149"/>
-      <c r="C8" s="147"/>
-      <c r="D8" s="147"/>
+      <c r="B8" s="153"/>
+      <c r="C8" s="156"/>
+      <c r="D8" s="156"/>
       <c r="E8" s="81"/>
       <c r="F8" s="92" t="s">
         <v>62</v>
@@ -3578,7 +3578,7 @@
         <v>100</v>
       </c>
       <c r="P8" s="90">
-        <v>11331</v>
+        <v>47856</v>
       </c>
       <c r="Q8" s="82"/>
       <c r="R8" s="82" t="s">
@@ -3631,17 +3631,17 @@
       <c r="AI8" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ8" s="149"/>
+      <c r="AJ8" s="153"/>
       <c r="AK8" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL8" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM8" s="149"/>
-      <c r="AN8" s="169"/>
-      <c r="AO8" s="169"/>
-      <c r="AP8" s="149"/>
+      <c r="AM8" s="153"/>
+      <c r="AN8" s="163"/>
+      <c r="AO8" s="163"/>
+      <c r="AP8" s="153"/>
       <c r="AQ8" s="92" t="s">
         <v>92</v>
       </c>
@@ -3714,13 +3714,13 @@
       <c r="A9" s="26">
         <v>1</v>
       </c>
-      <c r="B9" s="172" t="s">
+      <c r="B9" s="147" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="174" t="s">
+      <c r="C9" s="149" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="174" t="s">
+      <c r="D9" s="149" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="26"/>
@@ -3808,7 +3808,7 @@
       <c r="AI9" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="AJ9" s="172">
+      <c r="AJ9" s="147">
         <v>1</v>
       </c>
       <c r="AK9" s="141" t="s">
@@ -3817,16 +3817,16 @@
       <c r="AL9" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM9" s="165" t="s">
+      <c r="AM9" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="AN9" s="163">
+      <c r="AN9" s="143">
         <v>46120</v>
       </c>
-      <c r="AO9" s="163">
+      <c r="AO9" s="143">
         <v>46126</v>
       </c>
-      <c r="AP9" s="165">
+      <c r="AP9" s="145">
         <v>6</v>
       </c>
       <c r="AQ9" s="52" t="s">
@@ -3898,9 +3898,9 @@
       <c r="A10" s="45">
         <v>2</v>
       </c>
-      <c r="B10" s="173"/>
-      <c r="C10" s="175"/>
-      <c r="D10" s="175"/>
+      <c r="B10" s="148"/>
+      <c r="C10" s="150"/>
+      <c r="D10" s="150"/>
       <c r="E10" s="45"/>
       <c r="F10" s="48" t="s">
         <v>62</v>
@@ -3982,17 +3982,17 @@
       <c r="AI10" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="AJ10" s="173"/>
+      <c r="AJ10" s="148"/>
       <c r="AK10" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL10" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM10" s="166"/>
-      <c r="AN10" s="164"/>
-      <c r="AO10" s="164"/>
-      <c r="AP10" s="166"/>
+      <c r="AM10" s="146"/>
+      <c r="AN10" s="144"/>
+      <c r="AO10" s="144"/>
+      <c r="AP10" s="146"/>
       <c r="AQ10" s="48" t="s">
         <v>111</v>
       </c>
@@ -4062,13 +4062,13 @@
       <c r="A11" s="26">
         <v>1</v>
       </c>
-      <c r="B11" s="172" t="s">
+      <c r="B11" s="147" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="174" t="s">
+      <c r="C11" s="149" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="174" t="s">
+      <c r="D11" s="149" t="s">
         <v>61</v>
       </c>
       <c r="E11" s="26"/>
@@ -4132,7 +4132,7 @@
       <c r="AI11" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="AJ11" s="172">
+      <c r="AJ11" s="147">
         <v>1</v>
       </c>
       <c r="AK11" s="141" t="s">
@@ -4141,16 +4141,16 @@
       <c r="AL11" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM11" s="165" t="s">
+      <c r="AM11" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="AN11" s="163">
+      <c r="AN11" s="143">
         <v>46132</v>
       </c>
-      <c r="AO11" s="163">
+      <c r="AO11" s="143">
         <v>46138</v>
       </c>
-      <c r="AP11" s="165">
+      <c r="AP11" s="145">
         <v>6</v>
       </c>
       <c r="AQ11" s="52" t="s">
@@ -4204,9 +4204,9 @@
       <c r="A12" s="45">
         <v>2</v>
       </c>
-      <c r="B12" s="173"/>
-      <c r="C12" s="175"/>
-      <c r="D12" s="175"/>
+      <c r="B12" s="148"/>
+      <c r="C12" s="150"/>
+      <c r="D12" s="150"/>
       <c r="E12" s="45"/>
       <c r="F12" s="48" t="s">
         <v>62</v>
@@ -4268,17 +4268,17 @@
       <c r="AI12" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="AJ12" s="173"/>
+      <c r="AJ12" s="148"/>
       <c r="AK12" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL12" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM12" s="166"/>
-      <c r="AN12" s="164"/>
-      <c r="AO12" s="164"/>
-      <c r="AP12" s="166"/>
+      <c r="AM12" s="146"/>
+      <c r="AN12" s="144"/>
+      <c r="AO12" s="144"/>
+      <c r="AP12" s="146"/>
       <c r="AQ12" s="48" t="s">
         <v>122</v>
       </c>
@@ -9202,33 +9202,6 @@
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AM11:AM12"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="AJ9:AJ10"/>
-    <mergeCell ref="AM9:AM10"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="AJ6:AJ8"/>
-    <mergeCell ref="AM6:AM8"/>
-    <mergeCell ref="AJ2:AP2"/>
-    <mergeCell ref="V2:AB2"/>
-    <mergeCell ref="AC2:AI2"/>
-    <mergeCell ref="AN9:AN10"/>
-    <mergeCell ref="AO9:AO10"/>
-    <mergeCell ref="AP9:AP10"/>
-    <mergeCell ref="AN6:AN8"/>
-    <mergeCell ref="AO6:AO8"/>
-    <mergeCell ref="AP6:AP8"/>
     <mergeCell ref="B1:BQ1"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="C4:C5"/>
@@ -9245,6 +9218,33 @@
     <mergeCell ref="BI2:BQ2"/>
     <mergeCell ref="G2:U2"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="AJ2:AP2"/>
+    <mergeCell ref="V2:AB2"/>
+    <mergeCell ref="AC2:AI2"/>
+    <mergeCell ref="AN9:AN10"/>
+    <mergeCell ref="AO9:AO10"/>
+    <mergeCell ref="AP9:AP10"/>
+    <mergeCell ref="AN6:AN8"/>
+    <mergeCell ref="AO6:AO8"/>
+    <mergeCell ref="AP6:AP8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="AJ6:AJ8"/>
+    <mergeCell ref="AM6:AM8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="AJ9:AJ10"/>
+    <mergeCell ref="AM9:AM10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AM11:AM12"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
@@ -9271,15 +9271,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005310FD7AD7CB004A8A6A0F373B4D2C9A" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e03df01192bc7a0d3daab74abc4d5196">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6400beab-f54b-4fe2-8a3b-8916a6012868" xmlns:ns3="af8b05c0-1ee2-463e-b79d-b3491b282b4f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c21e3be90755f8fba129abf768e1fac6" ns2:_="" ns3:_="">
     <xsd:import namespace="6400beab-f54b-4fe2-8a3b-8916a6012868"/>
@@ -9540,6 +9531,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{515C1B63-7175-4E1B-B42F-E31C07EF7985}">
   <ds:schemaRefs>
@@ -9558,14 +9558,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01D4BAD6-B1CF-44C3-8924-5E31C0B35D19}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9582,4 +9574,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
manual hotel logo registry working with fallback and correct path resolution
</commit_message>
<xml_diff>
--- a/voucher_generator/LISTADO GENERAL - MODELO.xlsx
+++ b/voucher_generator/LISTADO GENERAL - MODELO.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ignac\Desktop\sharepoint_pipeline_app\voucher_generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\sharepoint_pipeline_app\voucher_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724D405A-79FB-4FEF-9806-72E2199449F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{796B918A-1E23-46E2-B6F6-8069CC5C18B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" xr2:uid="{E92A6B87-369E-48A6-A293-58A76914B5E4}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="134">
   <si>
     <t>NOMBRE DEL EVENTO Y CANTIDAD DE PAX</t>
   </si>
@@ -474,6 +474,15 @@
   </si>
   <si>
     <t xml:space="preserve">Punta Cana </t>
+  </si>
+  <si>
+    <t>NEW YORK CITY</t>
+  </si>
+  <si>
+    <t>New York City</t>
+  </si>
+  <si>
+    <t>World Center Hotel</t>
   </si>
 </sst>
 </file>
@@ -1423,6 +1432,66 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="12" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="16" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1435,6 +1504,21 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1446,81 +1530,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="12" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1914,76 +1923,76 @@
   <sheetData>
     <row r="1" spans="1:149" ht="12.75" customHeight="1">
       <c r="A1" s="38"/>
-      <c r="B1" s="164" t="s">
+      <c r="B1" s="143" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
-      <c r="G1" s="157"/>
-      <c r="H1" s="157"/>
-      <c r="I1" s="157"/>
-      <c r="J1" s="157"/>
-      <c r="K1" s="157"/>
-      <c r="L1" s="157"/>
-      <c r="M1" s="157"/>
-      <c r="N1" s="157"/>
-      <c r="O1" s="157"/>
-      <c r="P1" s="157"/>
-      <c r="Q1" s="157"/>
-      <c r="R1" s="157"/>
-      <c r="S1" s="157"/>
-      <c r="T1" s="157"/>
-      <c r="U1" s="157"/>
-      <c r="V1" s="157"/>
-      <c r="W1" s="157"/>
-      <c r="X1" s="157"/>
-      <c r="Y1" s="157"/>
-      <c r="Z1" s="157"/>
-      <c r="AA1" s="157"/>
-      <c r="AB1" s="157"/>
-      <c r="AC1" s="157"/>
-      <c r="AD1" s="157"/>
-      <c r="AE1" s="157"/>
-      <c r="AF1" s="157"/>
-      <c r="AG1" s="157"/>
-      <c r="AH1" s="157"/>
-      <c r="AI1" s="157"/>
-      <c r="AJ1" s="157"/>
-      <c r="AK1" s="157"/>
-      <c r="AL1" s="157"/>
-      <c r="AM1" s="157"/>
-      <c r="AN1" s="157"/>
-      <c r="AO1" s="157"/>
-      <c r="AP1" s="157"/>
-      <c r="AQ1" s="157"/>
-      <c r="AR1" s="157"/>
-      <c r="AS1" s="157"/>
-      <c r="AT1" s="157"/>
-      <c r="AU1" s="157"/>
-      <c r="AV1" s="157"/>
-      <c r="AW1" s="157"/>
-      <c r="AX1" s="157"/>
-      <c r="AY1" s="157"/>
-      <c r="AZ1" s="157"/>
-      <c r="BA1" s="157"/>
-      <c r="BB1" s="157"/>
-      <c r="BC1" s="157"/>
-      <c r="BD1" s="157"/>
-      <c r="BE1" s="157"/>
-      <c r="BF1" s="157"/>
-      <c r="BG1" s="157"/>
-      <c r="BH1" s="157"/>
-      <c r="BI1" s="157"/>
-      <c r="BJ1" s="157"/>
-      <c r="BK1" s="157"/>
-      <c r="BL1" s="157"/>
-      <c r="BM1" s="157"/>
-      <c r="BN1" s="157"/>
-      <c r="BO1" s="157"/>
-      <c r="BP1" s="157"/>
-      <c r="BQ1" s="165"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
+      <c r="J1" s="144"/>
+      <c r="K1" s="144"/>
+      <c r="L1" s="144"/>
+      <c r="M1" s="144"/>
+      <c r="N1" s="144"/>
+      <c r="O1" s="144"/>
+      <c r="P1" s="144"/>
+      <c r="Q1" s="144"/>
+      <c r="R1" s="144"/>
+      <c r="S1" s="144"/>
+      <c r="T1" s="144"/>
+      <c r="U1" s="144"/>
+      <c r="V1" s="144"/>
+      <c r="W1" s="144"/>
+      <c r="X1" s="144"/>
+      <c r="Y1" s="144"/>
+      <c r="Z1" s="144"/>
+      <c r="AA1" s="144"/>
+      <c r="AB1" s="144"/>
+      <c r="AC1" s="144"/>
+      <c r="AD1" s="144"/>
+      <c r="AE1" s="144"/>
+      <c r="AF1" s="144"/>
+      <c r="AG1" s="144"/>
+      <c r="AH1" s="144"/>
+      <c r="AI1" s="144"/>
+      <c r="AJ1" s="144"/>
+      <c r="AK1" s="144"/>
+      <c r="AL1" s="144"/>
+      <c r="AM1" s="144"/>
+      <c r="AN1" s="144"/>
+      <c r="AO1" s="144"/>
+      <c r="AP1" s="144"/>
+      <c r="AQ1" s="144"/>
+      <c r="AR1" s="144"/>
+      <c r="AS1" s="144"/>
+      <c r="AT1" s="144"/>
+      <c r="AU1" s="144"/>
+      <c r="AV1" s="144"/>
+      <c r="AW1" s="144"/>
+      <c r="AX1" s="144"/>
+      <c r="AY1" s="144"/>
+      <c r="AZ1" s="144"/>
+      <c r="BA1" s="144"/>
+      <c r="BB1" s="144"/>
+      <c r="BC1" s="144"/>
+      <c r="BD1" s="144"/>
+      <c r="BE1" s="144"/>
+      <c r="BF1" s="144"/>
+      <c r="BG1" s="144"/>
+      <c r="BH1" s="144"/>
+      <c r="BI1" s="144"/>
+      <c r="BJ1" s="144"/>
+      <c r="BK1" s="144"/>
+      <c r="BL1" s="144"/>
+      <c r="BM1" s="144"/>
+      <c r="BN1" s="144"/>
+      <c r="BO1" s="144"/>
+      <c r="BP1" s="144"/>
+      <c r="BQ1" s="145"/>
       <c r="BR1" s="20"/>
       <c r="BS1" s="20"/>
       <c r="BT1" s="20"/>
@@ -2067,98 +2076,98 @@
     </row>
     <row r="2" spans="1:149" ht="15" customHeight="1">
       <c r="A2" s="39"/>
-      <c r="B2" s="171" t="s">
+      <c r="B2" s="157" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="175"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="161"/>
       <c r="E2" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="170" t="s">
+      <c r="G2" s="156" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
-      <c r="O2" s="171"/>
-      <c r="P2" s="171"/>
-      <c r="Q2" s="171"/>
-      <c r="R2" s="171"/>
-      <c r="S2" s="171"/>
-      <c r="T2" s="171"/>
-      <c r="U2" s="175"/>
-      <c r="V2" s="158" t="s">
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
+      <c r="M2" s="157"/>
+      <c r="N2" s="157"/>
+      <c r="O2" s="157"/>
+      <c r="P2" s="157"/>
+      <c r="Q2" s="157"/>
+      <c r="R2" s="157"/>
+      <c r="S2" s="157"/>
+      <c r="T2" s="157"/>
+      <c r="U2" s="161"/>
+      <c r="V2" s="153" t="s">
         <v>5</v>
       </c>
-      <c r="W2" s="158"/>
-      <c r="X2" s="158"/>
-      <c r="Y2" s="158"/>
-      <c r="Z2" s="158"/>
-      <c r="AA2" s="158"/>
-      <c r="AB2" s="158"/>
-      <c r="AC2" s="159" t="s">
+      <c r="W2" s="153"/>
+      <c r="X2" s="153"/>
+      <c r="Y2" s="153"/>
+      <c r="Z2" s="153"/>
+      <c r="AA2" s="153"/>
+      <c r="AB2" s="153"/>
+      <c r="AC2" s="152" t="s">
         <v>6</v>
       </c>
-      <c r="AD2" s="158"/>
-      <c r="AE2" s="158"/>
-      <c r="AF2" s="158"/>
-      <c r="AG2" s="158"/>
-      <c r="AH2" s="158"/>
-      <c r="AI2" s="160"/>
-      <c r="AJ2" s="157" t="s">
+      <c r="AD2" s="153"/>
+      <c r="AE2" s="153"/>
+      <c r="AF2" s="153"/>
+      <c r="AG2" s="153"/>
+      <c r="AH2" s="153"/>
+      <c r="AI2" s="162"/>
+      <c r="AJ2" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="AK2" s="157"/>
-      <c r="AL2" s="157"/>
-      <c r="AM2" s="157"/>
-      <c r="AN2" s="157"/>
-      <c r="AO2" s="157"/>
-      <c r="AP2" s="157"/>
-      <c r="AQ2" s="159" t="s">
+      <c r="AK2" s="144"/>
+      <c r="AL2" s="144"/>
+      <c r="AM2" s="144"/>
+      <c r="AN2" s="144"/>
+      <c r="AO2" s="144"/>
+      <c r="AP2" s="144"/>
+      <c r="AQ2" s="152" t="s">
         <v>8</v>
       </c>
-      <c r="AR2" s="158"/>
-      <c r="AS2" s="158"/>
-      <c r="AT2" s="158"/>
-      <c r="AU2" s="158"/>
-      <c r="AV2" s="158"/>
-      <c r="AW2" s="158"/>
-      <c r="AX2" s="159" t="s">
+      <c r="AR2" s="153"/>
+      <c r="AS2" s="153"/>
+      <c r="AT2" s="153"/>
+      <c r="AU2" s="153"/>
+      <c r="AV2" s="153"/>
+      <c r="AW2" s="153"/>
+      <c r="AX2" s="152" t="s">
         <v>9</v>
       </c>
-      <c r="AY2" s="158"/>
-      <c r="AZ2" s="158"/>
-      <c r="BA2" s="158"/>
-      <c r="BB2" s="158"/>
-      <c r="BC2" s="158"/>
-      <c r="BD2" s="158"/>
-      <c r="BE2" s="168" t="s">
+      <c r="AY2" s="153"/>
+      <c r="AZ2" s="153"/>
+      <c r="BA2" s="153"/>
+      <c r="BB2" s="153"/>
+      <c r="BC2" s="153"/>
+      <c r="BD2" s="153"/>
+      <c r="BE2" s="154" t="s">
         <v>2</v>
       </c>
-      <c r="BF2" s="169"/>
-      <c r="BG2" s="170" t="s">
+      <c r="BF2" s="155"/>
+      <c r="BG2" s="156" t="s">
         <v>10</v>
       </c>
-      <c r="BH2" s="171"/>
-      <c r="BI2" s="172" t="s">
+      <c r="BH2" s="157"/>
+      <c r="BI2" s="158" t="s">
         <v>11</v>
       </c>
-      <c r="BJ2" s="173"/>
-      <c r="BK2" s="173"/>
-      <c r="BL2" s="173"/>
-      <c r="BM2" s="173"/>
-      <c r="BN2" s="173"/>
-      <c r="BO2" s="173"/>
-      <c r="BP2" s="173"/>
-      <c r="BQ2" s="174"/>
+      <c r="BJ2" s="159"/>
+      <c r="BK2" s="159"/>
+      <c r="BL2" s="159"/>
+      <c r="BM2" s="159"/>
+      <c r="BN2" s="159"/>
+      <c r="BO2" s="159"/>
+      <c r="BP2" s="159"/>
+      <c r="BQ2" s="160"/>
       <c r="BR2" s="20"/>
       <c r="BS2" s="20"/>
       <c r="BT2" s="20"/>
@@ -2533,13 +2542,13 @@
       <c r="A4" s="68">
         <v>1</v>
       </c>
-      <c r="B4" s="152" t="s">
+      <c r="B4" s="148" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="155" t="s">
+      <c r="C4" s="146" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="155" t="s">
+      <c r="D4" s="146" t="s">
         <v>61</v>
       </c>
       <c r="E4" s="68"/>
@@ -2619,7 +2628,7 @@
       <c r="AI4" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ4" s="166">
+      <c r="AJ4" s="150">
         <v>1</v>
       </c>
       <c r="AK4" s="141" t="s">
@@ -2628,16 +2637,16 @@
       <c r="AL4" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM4" s="166" t="s">
+      <c r="AM4" s="150" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="167">
+      <c r="AN4" s="151">
         <v>45709</v>
       </c>
-      <c r="AO4" s="167">
+      <c r="AO4" s="151">
         <v>45715</v>
       </c>
-      <c r="AP4" s="166">
+      <c r="AP4" s="150">
         <v>6</v>
       </c>
       <c r="AQ4" s="69" t="s">
@@ -2798,9 +2807,9 @@
       <c r="A5" s="81">
         <v>2</v>
       </c>
-      <c r="B5" s="153"/>
-      <c r="C5" s="156"/>
-      <c r="D5" s="156"/>
+      <c r="B5" s="149"/>
+      <c r="C5" s="147"/>
+      <c r="D5" s="147"/>
       <c r="E5" s="81"/>
       <c r="F5" s="82" t="s">
         <v>62</v>
@@ -2870,17 +2879,17 @@
       <c r="AI5" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ5" s="153"/>
+      <c r="AJ5" s="149"/>
       <c r="AK5" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL5" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM5" s="153"/>
-      <c r="AN5" s="153"/>
-      <c r="AO5" s="153"/>
-      <c r="AP5" s="153"/>
+      <c r="AM5" s="149"/>
+      <c r="AN5" s="149"/>
+      <c r="AO5" s="149"/>
+      <c r="AP5" s="149"/>
       <c r="AQ5" s="82" t="s">
         <v>75</v>
       </c>
@@ -3039,13 +3048,13 @@
       <c r="A6" s="110">
         <v>1</v>
       </c>
-      <c r="B6" s="151" t="s">
+      <c r="B6" s="170" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="154" t="s">
+      <c r="C6" s="171" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="154" t="s">
+      <c r="D6" s="171" t="s">
         <v>61</v>
       </c>
       <c r="E6" s="110"/>
@@ -3131,7 +3140,7 @@
       <c r="AI6" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ6" s="151">
+      <c r="AJ6" s="170">
         <v>1</v>
       </c>
       <c r="AK6" s="141" t="s">
@@ -3140,16 +3149,16 @@
       <c r="AL6" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM6" s="151" t="s">
+      <c r="AM6" s="170" t="s">
         <v>74</v>
       </c>
-      <c r="AN6" s="161">
+      <c r="AN6" s="167">
         <v>46104</v>
       </c>
-      <c r="AO6" s="161">
+      <c r="AO6" s="167">
         <v>46110</v>
       </c>
-      <c r="AP6" s="151">
+      <c r="AP6" s="170">
         <v>6</v>
       </c>
       <c r="AQ6" s="111" t="s">
@@ -3304,9 +3313,9 @@
       <c r="A7" s="125">
         <v>2</v>
       </c>
-      <c r="B7" s="152"/>
-      <c r="C7" s="155"/>
-      <c r="D7" s="155"/>
+      <c r="B7" s="148"/>
+      <c r="C7" s="146"/>
+      <c r="D7" s="146"/>
       <c r="E7" s="125"/>
       <c r="F7" s="111" t="s">
         <v>62</v>
@@ -3386,17 +3395,17 @@
       <c r="AI7" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ7" s="152"/>
+      <c r="AJ7" s="148"/>
       <c r="AK7" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL7" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM7" s="152"/>
-      <c r="AN7" s="162"/>
-      <c r="AO7" s="162"/>
-      <c r="AP7" s="152"/>
+      <c r="AM7" s="148"/>
+      <c r="AN7" s="168"/>
+      <c r="AO7" s="168"/>
+      <c r="AP7" s="148"/>
       <c r="AQ7" s="111" t="s">
         <v>92</v>
       </c>
@@ -3549,9 +3558,9 @@
       <c r="A8" s="81">
         <v>3</v>
       </c>
-      <c r="B8" s="153"/>
-      <c r="C8" s="156"/>
-      <c r="D8" s="156"/>
+      <c r="B8" s="149"/>
+      <c r="C8" s="147"/>
+      <c r="D8" s="147"/>
       <c r="E8" s="81"/>
       <c r="F8" s="92" t="s">
         <v>62</v>
@@ -3631,17 +3640,17 @@
       <c r="AI8" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ8" s="153"/>
+      <c r="AJ8" s="149"/>
       <c r="AK8" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL8" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM8" s="153"/>
-      <c r="AN8" s="163"/>
-      <c r="AO8" s="163"/>
-      <c r="AP8" s="153"/>
+      <c r="AM8" s="149"/>
+      <c r="AN8" s="169"/>
+      <c r="AO8" s="169"/>
+      <c r="AP8" s="149"/>
       <c r="AQ8" s="92" t="s">
         <v>92</v>
       </c>
@@ -3714,18 +3723,18 @@
       <c r="A9" s="26">
         <v>1</v>
       </c>
-      <c r="B9" s="147" t="s">
+      <c r="B9" s="172" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="149" t="s">
+      <c r="C9" s="174" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="149" t="s">
+      <c r="D9" s="174" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="26"/>
       <c r="F9" s="52" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="G9" s="57" t="s">
         <v>101</v>
@@ -3808,25 +3817,25 @@
       <c r="AI9" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="AJ9" s="147">
+      <c r="AJ9" s="172">
         <v>1</v>
       </c>
       <c r="AK9" s="141" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AL9" s="141" t="s">
-        <v>128</v>
-      </c>
-      <c r="AM9" s="145" t="s">
+        <v>133</v>
+      </c>
+      <c r="AM9" s="165" t="s">
         <v>74</v>
       </c>
-      <c r="AN9" s="143">
+      <c r="AN9" s="163">
         <v>46120</v>
       </c>
-      <c r="AO9" s="143">
+      <c r="AO9" s="163">
         <v>46126</v>
       </c>
-      <c r="AP9" s="145">
+      <c r="AP9" s="165">
         <v>6</v>
       </c>
       <c r="AQ9" s="52" t="s">
@@ -3898,12 +3907,12 @@
       <c r="A10" s="45">
         <v>2</v>
       </c>
-      <c r="B10" s="148"/>
-      <c r="C10" s="150"/>
-      <c r="D10" s="150"/>
+      <c r="B10" s="173"/>
+      <c r="C10" s="175"/>
+      <c r="D10" s="175"/>
       <c r="E10" s="45"/>
-      <c r="F10" s="48" t="s">
-        <v>62</v>
+      <c r="F10" s="52" t="s">
+        <v>131</v>
       </c>
       <c r="G10" s="58" t="s">
         <v>113</v>
@@ -3982,17 +3991,17 @@
       <c r="AI10" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="AJ10" s="148"/>
+      <c r="AJ10" s="173"/>
       <c r="AK10" s="141" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AL10" s="141" t="s">
-        <v>128</v>
-      </c>
-      <c r="AM10" s="146"/>
-      <c r="AN10" s="144"/>
-      <c r="AO10" s="144"/>
-      <c r="AP10" s="146"/>
+        <v>133</v>
+      </c>
+      <c r="AM10" s="166"/>
+      <c r="AN10" s="164"/>
+      <c r="AO10" s="164"/>
+      <c r="AP10" s="166"/>
       <c r="AQ10" s="48" t="s">
         <v>111</v>
       </c>
@@ -4062,13 +4071,13 @@
       <c r="A11" s="26">
         <v>1</v>
       </c>
-      <c r="B11" s="147" t="s">
+      <c r="B11" s="172" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="149" t="s">
+      <c r="C11" s="174" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="149" t="s">
+      <c r="D11" s="174" t="s">
         <v>61</v>
       </c>
       <c r="E11" s="26"/>
@@ -4132,7 +4141,7 @@
       <c r="AI11" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="AJ11" s="147">
+      <c r="AJ11" s="172">
         <v>1</v>
       </c>
       <c r="AK11" s="141" t="s">
@@ -4141,16 +4150,16 @@
       <c r="AL11" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM11" s="145" t="s">
+      <c r="AM11" s="165" t="s">
         <v>74</v>
       </c>
-      <c r="AN11" s="143">
+      <c r="AN11" s="163">
         <v>46132</v>
       </c>
-      <c r="AO11" s="143">
+      <c r="AO11" s="163">
         <v>46138</v>
       </c>
-      <c r="AP11" s="145">
+      <c r="AP11" s="165">
         <v>6</v>
       </c>
       <c r="AQ11" s="52" t="s">
@@ -4204,9 +4213,9 @@
       <c r="A12" s="45">
         <v>2</v>
       </c>
-      <c r="B12" s="148"/>
-      <c r="C12" s="150"/>
-      <c r="D12" s="150"/>
+      <c r="B12" s="173"/>
+      <c r="C12" s="175"/>
+      <c r="D12" s="175"/>
       <c r="E12" s="45"/>
       <c r="F12" s="48" t="s">
         <v>62</v>
@@ -4268,17 +4277,17 @@
       <c r="AI12" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="AJ12" s="148"/>
+      <c r="AJ12" s="173"/>
       <c r="AK12" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL12" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM12" s="146"/>
-      <c r="AN12" s="144"/>
-      <c r="AO12" s="144"/>
-      <c r="AP12" s="146"/>
+      <c r="AM12" s="166"/>
+      <c r="AN12" s="164"/>
+      <c r="AO12" s="164"/>
+      <c r="AP12" s="166"/>
       <c r="AQ12" s="48" t="s">
         <v>122</v>
       </c>
@@ -9202,6 +9211,33 @@
     </row>
   </sheetData>
   <mergeCells count="43">
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AM11:AM12"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="AJ9:AJ10"/>
+    <mergeCell ref="AM9:AM10"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="AJ6:AJ8"/>
+    <mergeCell ref="AM6:AM8"/>
+    <mergeCell ref="AJ2:AP2"/>
+    <mergeCell ref="V2:AB2"/>
+    <mergeCell ref="AC2:AI2"/>
+    <mergeCell ref="AN9:AN10"/>
+    <mergeCell ref="AO9:AO10"/>
+    <mergeCell ref="AP9:AP10"/>
+    <mergeCell ref="AN6:AN8"/>
+    <mergeCell ref="AO6:AO8"/>
+    <mergeCell ref="AP6:AP8"/>
     <mergeCell ref="B1:BQ1"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="C4:C5"/>
@@ -9218,33 +9254,6 @@
     <mergeCell ref="BI2:BQ2"/>
     <mergeCell ref="G2:U2"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="AJ2:AP2"/>
-    <mergeCell ref="V2:AB2"/>
-    <mergeCell ref="AC2:AI2"/>
-    <mergeCell ref="AN9:AN10"/>
-    <mergeCell ref="AO9:AO10"/>
-    <mergeCell ref="AP9:AP10"/>
-    <mergeCell ref="AN6:AN8"/>
-    <mergeCell ref="AO6:AO8"/>
-    <mergeCell ref="AP6:AP8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="AJ6:AJ8"/>
-    <mergeCell ref="AM6:AM8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="AJ9:AJ10"/>
-    <mergeCell ref="AM9:AM10"/>
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AM11:AM12"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
@@ -9271,6 +9280,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005310FD7AD7CB004A8A6A0F373B4D2C9A" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e03df01192bc7a0d3daab74abc4d5196">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6400beab-f54b-4fe2-8a3b-8916a6012868" xmlns:ns3="af8b05c0-1ee2-463e-b79d-b3491b282b4f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c21e3be90755f8fba129abf768e1fac6" ns2:_="" ns3:_="">
     <xsd:import namespace="6400beab-f54b-4fe2-8a3b-8916a6012868"/>
@@ -9531,15 +9549,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{515C1B63-7175-4E1B-B42F-E31C07EF7985}">
   <ds:schemaRefs>
@@ -9558,6 +9567,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01D4BAD6-B1CF-44C3-8924-5E31C0B35D19}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9574,12 +9591,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix hotel logo uploader flow and enrichment warnings pipeline result
</commit_message>
<xml_diff>
--- a/voucher_generator/LISTADO GENERAL - MODELO.xlsx
+++ b/voucher_generator/LISTADO GENERAL - MODELO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\sharepoint_pipeline_app\voucher_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{796B918A-1E23-46E2-B6F6-8069CC5C18B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22ED2F7-A583-449D-8BE6-483953E61224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" xr2:uid="{E92A6B87-369E-48A6-A293-58A76914B5E4}"/>
   </bookViews>
@@ -479,10 +479,10 @@
     <t>NEW YORK CITY</t>
   </si>
   <si>
+    <t>World Center Hotel</t>
+  </si>
+  <si>
     <t>New York City</t>
-  </si>
-  <si>
-    <t>World Center Hotel</t>
   </si>
 </sst>
 </file>
@@ -1432,39 +1432,81 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="12" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1488,48 +1530,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="2" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1923,76 +1923,76 @@
   <sheetData>
     <row r="1" spans="1:149" ht="12.75" customHeight="1">
       <c r="A1" s="38"/>
-      <c r="B1" s="143" t="s">
+      <c r="B1" s="164" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="144"/>
-      <c r="F1" s="144"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="144"/>
-      <c r="I1" s="144"/>
-      <c r="J1" s="144"/>
-      <c r="K1" s="144"/>
-      <c r="L1" s="144"/>
-      <c r="M1" s="144"/>
-      <c r="N1" s="144"/>
-      <c r="O1" s="144"/>
-      <c r="P1" s="144"/>
-      <c r="Q1" s="144"/>
-      <c r="R1" s="144"/>
-      <c r="S1" s="144"/>
-      <c r="T1" s="144"/>
-      <c r="U1" s="144"/>
-      <c r="V1" s="144"/>
-      <c r="W1" s="144"/>
-      <c r="X1" s="144"/>
-      <c r="Y1" s="144"/>
-      <c r="Z1" s="144"/>
-      <c r="AA1" s="144"/>
-      <c r="AB1" s="144"/>
-      <c r="AC1" s="144"/>
-      <c r="AD1" s="144"/>
-      <c r="AE1" s="144"/>
-      <c r="AF1" s="144"/>
-      <c r="AG1" s="144"/>
-      <c r="AH1" s="144"/>
-      <c r="AI1" s="144"/>
-      <c r="AJ1" s="144"/>
-      <c r="AK1" s="144"/>
-      <c r="AL1" s="144"/>
-      <c r="AM1" s="144"/>
-      <c r="AN1" s="144"/>
-      <c r="AO1" s="144"/>
-      <c r="AP1" s="144"/>
-      <c r="AQ1" s="144"/>
-      <c r="AR1" s="144"/>
-      <c r="AS1" s="144"/>
-      <c r="AT1" s="144"/>
-      <c r="AU1" s="144"/>
-      <c r="AV1" s="144"/>
-      <c r="AW1" s="144"/>
-      <c r="AX1" s="144"/>
-      <c r="AY1" s="144"/>
-      <c r="AZ1" s="144"/>
-      <c r="BA1" s="144"/>
-      <c r="BB1" s="144"/>
-      <c r="BC1" s="144"/>
-      <c r="BD1" s="144"/>
-      <c r="BE1" s="144"/>
-      <c r="BF1" s="144"/>
-      <c r="BG1" s="144"/>
-      <c r="BH1" s="144"/>
-      <c r="BI1" s="144"/>
-      <c r="BJ1" s="144"/>
-      <c r="BK1" s="144"/>
-      <c r="BL1" s="144"/>
-      <c r="BM1" s="144"/>
-      <c r="BN1" s="144"/>
-      <c r="BO1" s="144"/>
-      <c r="BP1" s="144"/>
-      <c r="BQ1" s="145"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
+      <c r="I1" s="157"/>
+      <c r="J1" s="157"/>
+      <c r="K1" s="157"/>
+      <c r="L1" s="157"/>
+      <c r="M1" s="157"/>
+      <c r="N1" s="157"/>
+      <c r="O1" s="157"/>
+      <c r="P1" s="157"/>
+      <c r="Q1" s="157"/>
+      <c r="R1" s="157"/>
+      <c r="S1" s="157"/>
+      <c r="T1" s="157"/>
+      <c r="U1" s="157"/>
+      <c r="V1" s="157"/>
+      <c r="W1" s="157"/>
+      <c r="X1" s="157"/>
+      <c r="Y1" s="157"/>
+      <c r="Z1" s="157"/>
+      <c r="AA1" s="157"/>
+      <c r="AB1" s="157"/>
+      <c r="AC1" s="157"/>
+      <c r="AD1" s="157"/>
+      <c r="AE1" s="157"/>
+      <c r="AF1" s="157"/>
+      <c r="AG1" s="157"/>
+      <c r="AH1" s="157"/>
+      <c r="AI1" s="157"/>
+      <c r="AJ1" s="157"/>
+      <c r="AK1" s="157"/>
+      <c r="AL1" s="157"/>
+      <c r="AM1" s="157"/>
+      <c r="AN1" s="157"/>
+      <c r="AO1" s="157"/>
+      <c r="AP1" s="157"/>
+      <c r="AQ1" s="157"/>
+      <c r="AR1" s="157"/>
+      <c r="AS1" s="157"/>
+      <c r="AT1" s="157"/>
+      <c r="AU1" s="157"/>
+      <c r="AV1" s="157"/>
+      <c r="AW1" s="157"/>
+      <c r="AX1" s="157"/>
+      <c r="AY1" s="157"/>
+      <c r="AZ1" s="157"/>
+      <c r="BA1" s="157"/>
+      <c r="BB1" s="157"/>
+      <c r="BC1" s="157"/>
+      <c r="BD1" s="157"/>
+      <c r="BE1" s="157"/>
+      <c r="BF1" s="157"/>
+      <c r="BG1" s="157"/>
+      <c r="BH1" s="157"/>
+      <c r="BI1" s="157"/>
+      <c r="BJ1" s="157"/>
+      <c r="BK1" s="157"/>
+      <c r="BL1" s="157"/>
+      <c r="BM1" s="157"/>
+      <c r="BN1" s="157"/>
+      <c r="BO1" s="157"/>
+      <c r="BP1" s="157"/>
+      <c r="BQ1" s="165"/>
       <c r="BR1" s="20"/>
       <c r="BS1" s="20"/>
       <c r="BT1" s="20"/>
@@ -2076,98 +2076,98 @@
     </row>
     <row r="2" spans="1:149" ht="15" customHeight="1">
       <c r="A2" s="39"/>
-      <c r="B2" s="157" t="s">
+      <c r="B2" s="171" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="157"/>
-      <c r="D2" s="161"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="175"/>
       <c r="E2" s="14" t="s">
         <v>2</v>
       </c>
       <c r="F2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="156" t="s">
+      <c r="G2" s="170" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="157"/>
-      <c r="N2" s="157"/>
-      <c r="O2" s="157"/>
-      <c r="P2" s="157"/>
-      <c r="Q2" s="157"/>
-      <c r="R2" s="157"/>
-      <c r="S2" s="157"/>
-      <c r="T2" s="157"/>
-      <c r="U2" s="161"/>
-      <c r="V2" s="153" t="s">
+      <c r="H2" s="171"/>
+      <c r="I2" s="171"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="171"/>
+      <c r="L2" s="171"/>
+      <c r="M2" s="171"/>
+      <c r="N2" s="171"/>
+      <c r="O2" s="171"/>
+      <c r="P2" s="171"/>
+      <c r="Q2" s="171"/>
+      <c r="R2" s="171"/>
+      <c r="S2" s="171"/>
+      <c r="T2" s="171"/>
+      <c r="U2" s="175"/>
+      <c r="V2" s="158" t="s">
         <v>5</v>
       </c>
-      <c r="W2" s="153"/>
-      <c r="X2" s="153"/>
-      <c r="Y2" s="153"/>
-      <c r="Z2" s="153"/>
-      <c r="AA2" s="153"/>
-      <c r="AB2" s="153"/>
-      <c r="AC2" s="152" t="s">
+      <c r="W2" s="158"/>
+      <c r="X2" s="158"/>
+      <c r="Y2" s="158"/>
+      <c r="Z2" s="158"/>
+      <c r="AA2" s="158"/>
+      <c r="AB2" s="158"/>
+      <c r="AC2" s="159" t="s">
         <v>6</v>
       </c>
-      <c r="AD2" s="153"/>
-      <c r="AE2" s="153"/>
-      <c r="AF2" s="153"/>
-      <c r="AG2" s="153"/>
-      <c r="AH2" s="153"/>
-      <c r="AI2" s="162"/>
-      <c r="AJ2" s="144" t="s">
+      <c r="AD2" s="158"/>
+      <c r="AE2" s="158"/>
+      <c r="AF2" s="158"/>
+      <c r="AG2" s="158"/>
+      <c r="AH2" s="158"/>
+      <c r="AI2" s="160"/>
+      <c r="AJ2" s="157" t="s">
         <v>7</v>
       </c>
-      <c r="AK2" s="144"/>
-      <c r="AL2" s="144"/>
-      <c r="AM2" s="144"/>
-      <c r="AN2" s="144"/>
-      <c r="AO2" s="144"/>
-      <c r="AP2" s="144"/>
-      <c r="AQ2" s="152" t="s">
+      <c r="AK2" s="157"/>
+      <c r="AL2" s="157"/>
+      <c r="AM2" s="157"/>
+      <c r="AN2" s="157"/>
+      <c r="AO2" s="157"/>
+      <c r="AP2" s="157"/>
+      <c r="AQ2" s="159" t="s">
         <v>8</v>
       </c>
-      <c r="AR2" s="153"/>
-      <c r="AS2" s="153"/>
-      <c r="AT2" s="153"/>
-      <c r="AU2" s="153"/>
-      <c r="AV2" s="153"/>
-      <c r="AW2" s="153"/>
-      <c r="AX2" s="152" t="s">
+      <c r="AR2" s="158"/>
+      <c r="AS2" s="158"/>
+      <c r="AT2" s="158"/>
+      <c r="AU2" s="158"/>
+      <c r="AV2" s="158"/>
+      <c r="AW2" s="158"/>
+      <c r="AX2" s="159" t="s">
         <v>9</v>
       </c>
-      <c r="AY2" s="153"/>
-      <c r="AZ2" s="153"/>
-      <c r="BA2" s="153"/>
-      <c r="BB2" s="153"/>
-      <c r="BC2" s="153"/>
-      <c r="BD2" s="153"/>
-      <c r="BE2" s="154" t="s">
+      <c r="AY2" s="158"/>
+      <c r="AZ2" s="158"/>
+      <c r="BA2" s="158"/>
+      <c r="BB2" s="158"/>
+      <c r="BC2" s="158"/>
+      <c r="BD2" s="158"/>
+      <c r="BE2" s="168" t="s">
         <v>2</v>
       </c>
-      <c r="BF2" s="155"/>
-      <c r="BG2" s="156" t="s">
+      <c r="BF2" s="169"/>
+      <c r="BG2" s="170" t="s">
         <v>10</v>
       </c>
-      <c r="BH2" s="157"/>
-      <c r="BI2" s="158" t="s">
+      <c r="BH2" s="171"/>
+      <c r="BI2" s="172" t="s">
         <v>11</v>
       </c>
-      <c r="BJ2" s="159"/>
-      <c r="BK2" s="159"/>
-      <c r="BL2" s="159"/>
-      <c r="BM2" s="159"/>
-      <c r="BN2" s="159"/>
-      <c r="BO2" s="159"/>
-      <c r="BP2" s="159"/>
-      <c r="BQ2" s="160"/>
+      <c r="BJ2" s="173"/>
+      <c r="BK2" s="173"/>
+      <c r="BL2" s="173"/>
+      <c r="BM2" s="173"/>
+      <c r="BN2" s="173"/>
+      <c r="BO2" s="173"/>
+      <c r="BP2" s="173"/>
+      <c r="BQ2" s="174"/>
       <c r="BR2" s="20"/>
       <c r="BS2" s="20"/>
       <c r="BT2" s="20"/>
@@ -2542,13 +2542,13 @@
       <c r="A4" s="68">
         <v>1</v>
       </c>
-      <c r="B4" s="148" t="s">
+      <c r="B4" s="152" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="146" t="s">
+      <c r="C4" s="155" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="146" t="s">
+      <c r="D4" s="155" t="s">
         <v>61</v>
       </c>
       <c r="E4" s="68"/>
@@ -2628,7 +2628,7 @@
       <c r="AI4" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ4" s="150">
+      <c r="AJ4" s="166">
         <v>1</v>
       </c>
       <c r="AK4" s="141" t="s">
@@ -2637,16 +2637,16 @@
       <c r="AL4" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM4" s="150" t="s">
+      <c r="AM4" s="166" t="s">
         <v>74</v>
       </c>
-      <c r="AN4" s="151">
+      <c r="AN4" s="167">
         <v>45709</v>
       </c>
-      <c r="AO4" s="151">
+      <c r="AO4" s="167">
         <v>45715</v>
       </c>
-      <c r="AP4" s="150">
+      <c r="AP4" s="166">
         <v>6</v>
       </c>
       <c r="AQ4" s="69" t="s">
@@ -2807,9 +2807,9 @@
       <c r="A5" s="81">
         <v>2</v>
       </c>
-      <c r="B5" s="149"/>
-      <c r="C5" s="147"/>
-      <c r="D5" s="147"/>
+      <c r="B5" s="153"/>
+      <c r="C5" s="156"/>
+      <c r="D5" s="156"/>
       <c r="E5" s="81"/>
       <c r="F5" s="82" t="s">
         <v>62</v>
@@ -2879,17 +2879,17 @@
       <c r="AI5" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ5" s="149"/>
+      <c r="AJ5" s="153"/>
       <c r="AK5" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL5" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM5" s="149"/>
-      <c r="AN5" s="149"/>
-      <c r="AO5" s="149"/>
-      <c r="AP5" s="149"/>
+      <c r="AM5" s="153"/>
+      <c r="AN5" s="153"/>
+      <c r="AO5" s="153"/>
+      <c r="AP5" s="153"/>
       <c r="AQ5" s="82" t="s">
         <v>75</v>
       </c>
@@ -3048,13 +3048,13 @@
       <c r="A6" s="110">
         <v>1</v>
       </c>
-      <c r="B6" s="170" t="s">
+      <c r="B6" s="151" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="171" t="s">
+      <c r="C6" s="154" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="171" t="s">
+      <c r="D6" s="154" t="s">
         <v>61</v>
       </c>
       <c r="E6" s="110"/>
@@ -3140,7 +3140,7 @@
       <c r="AI6" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ6" s="170">
+      <c r="AJ6" s="151">
         <v>1</v>
       </c>
       <c r="AK6" s="141" t="s">
@@ -3149,16 +3149,16 @@
       <c r="AL6" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM6" s="170" t="s">
+      <c r="AM6" s="151" t="s">
         <v>74</v>
       </c>
-      <c r="AN6" s="167">
+      <c r="AN6" s="161">
         <v>46104</v>
       </c>
-      <c r="AO6" s="167">
+      <c r="AO6" s="161">
         <v>46110</v>
       </c>
-      <c r="AP6" s="170">
+      <c r="AP6" s="151">
         <v>6</v>
       </c>
       <c r="AQ6" s="111" t="s">
@@ -3313,9 +3313,9 @@
       <c r="A7" s="125">
         <v>2</v>
       </c>
-      <c r="B7" s="148"/>
-      <c r="C7" s="146"/>
-      <c r="D7" s="146"/>
+      <c r="B7" s="152"/>
+      <c r="C7" s="155"/>
+      <c r="D7" s="155"/>
       <c r="E7" s="125"/>
       <c r="F7" s="111" t="s">
         <v>62</v>
@@ -3395,17 +3395,17 @@
       <c r="AI7" s="69" t="s">
         <v>73</v>
       </c>
-      <c r="AJ7" s="148"/>
+      <c r="AJ7" s="152"/>
       <c r="AK7" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL7" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM7" s="148"/>
-      <c r="AN7" s="168"/>
-      <c r="AO7" s="168"/>
-      <c r="AP7" s="148"/>
+      <c r="AM7" s="152"/>
+      <c r="AN7" s="162"/>
+      <c r="AO7" s="162"/>
+      <c r="AP7" s="152"/>
       <c r="AQ7" s="111" t="s">
         <v>92</v>
       </c>
@@ -3558,9 +3558,9 @@
       <c r="A8" s="81">
         <v>3</v>
       </c>
-      <c r="B8" s="149"/>
-      <c r="C8" s="147"/>
-      <c r="D8" s="147"/>
+      <c r="B8" s="153"/>
+      <c r="C8" s="156"/>
+      <c r="D8" s="156"/>
       <c r="E8" s="81"/>
       <c r="F8" s="92" t="s">
         <v>62</v>
@@ -3640,17 +3640,17 @@
       <c r="AI8" s="82" t="s">
         <v>73</v>
       </c>
-      <c r="AJ8" s="149"/>
+      <c r="AJ8" s="153"/>
       <c r="AK8" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL8" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM8" s="149"/>
-      <c r="AN8" s="169"/>
-      <c r="AO8" s="169"/>
-      <c r="AP8" s="149"/>
+      <c r="AM8" s="153"/>
+      <c r="AN8" s="163"/>
+      <c r="AO8" s="163"/>
+      <c r="AP8" s="153"/>
       <c r="AQ8" s="92" t="s">
         <v>92</v>
       </c>
@@ -3723,13 +3723,13 @@
       <c r="A9" s="26">
         <v>1</v>
       </c>
-      <c r="B9" s="172" t="s">
+      <c r="B9" s="147" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="174" t="s">
+      <c r="C9" s="149" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="174" t="s">
+      <c r="D9" s="149" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="26"/>
@@ -3817,25 +3817,25 @@
       <c r="AI9" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="AJ9" s="172">
+      <c r="AJ9" s="147">
         <v>1</v>
       </c>
       <c r="AK9" s="141" t="s">
+        <v>133</v>
+      </c>
+      <c r="AL9" s="141" t="s">
         <v>132</v>
       </c>
-      <c r="AL9" s="141" t="s">
-        <v>133</v>
-      </c>
-      <c r="AM9" s="165" t="s">
+      <c r="AM9" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="AN9" s="163">
+      <c r="AN9" s="143">
         <v>46120</v>
       </c>
-      <c r="AO9" s="163">
+      <c r="AO9" s="143">
         <v>46126</v>
       </c>
-      <c r="AP9" s="165">
+      <c r="AP9" s="145">
         <v>6</v>
       </c>
       <c r="AQ9" s="52" t="s">
@@ -3907,9 +3907,9 @@
       <c r="A10" s="45">
         <v>2</v>
       </c>
-      <c r="B10" s="173"/>
-      <c r="C10" s="175"/>
-      <c r="D10" s="175"/>
+      <c r="B10" s="148"/>
+      <c r="C10" s="150"/>
+      <c r="D10" s="150"/>
       <c r="E10" s="45"/>
       <c r="F10" s="52" t="s">
         <v>131</v>
@@ -3991,17 +3991,17 @@
       <c r="AI10" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="AJ10" s="173"/>
+      <c r="AJ10" s="148"/>
       <c r="AK10" s="141" t="s">
+        <v>133</v>
+      </c>
+      <c r="AL10" s="141" t="s">
         <v>132</v>
       </c>
-      <c r="AL10" s="141" t="s">
-        <v>133</v>
-      </c>
-      <c r="AM10" s="166"/>
-      <c r="AN10" s="164"/>
-      <c r="AO10" s="164"/>
-      <c r="AP10" s="166"/>
+      <c r="AM10" s="146"/>
+      <c r="AN10" s="144"/>
+      <c r="AO10" s="144"/>
+      <c r="AP10" s="146"/>
       <c r="AQ10" s="48" t="s">
         <v>111</v>
       </c>
@@ -4071,13 +4071,13 @@
       <c r="A11" s="26">
         <v>1</v>
       </c>
-      <c r="B11" s="172" t="s">
+      <c r="B11" s="147" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="174" t="s">
+      <c r="C11" s="149" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="174" t="s">
+      <c r="D11" s="149" t="s">
         <v>61</v>
       </c>
       <c r="E11" s="26"/>
@@ -4141,7 +4141,7 @@
       <c r="AI11" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="AJ11" s="172">
+      <c r="AJ11" s="147">
         <v>1</v>
       </c>
       <c r="AK11" s="141" t="s">
@@ -4150,16 +4150,16 @@
       <c r="AL11" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM11" s="165" t="s">
+      <c r="AM11" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="AN11" s="163">
+      <c r="AN11" s="143">
         <v>46132</v>
       </c>
-      <c r="AO11" s="163">
+      <c r="AO11" s="143">
         <v>46138</v>
       </c>
-      <c r="AP11" s="165">
+      <c r="AP11" s="145">
         <v>6</v>
       </c>
       <c r="AQ11" s="52" t="s">
@@ -4213,9 +4213,9 @@
       <c r="A12" s="45">
         <v>2</v>
       </c>
-      <c r="B12" s="173"/>
-      <c r="C12" s="175"/>
-      <c r="D12" s="175"/>
+      <c r="B12" s="148"/>
+      <c r="C12" s="150"/>
+      <c r="D12" s="150"/>
       <c r="E12" s="45"/>
       <c r="F12" s="48" t="s">
         <v>62</v>
@@ -4277,17 +4277,17 @@
       <c r="AI12" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="AJ12" s="173"/>
+      <c r="AJ12" s="148"/>
       <c r="AK12" s="141" t="s">
         <v>130</v>
       </c>
       <c r="AL12" s="141" t="s">
         <v>128</v>
       </c>
-      <c r="AM12" s="166"/>
-      <c r="AN12" s="164"/>
-      <c r="AO12" s="164"/>
-      <c r="AP12" s="166"/>
+      <c r="AM12" s="146"/>
+      <c r="AN12" s="144"/>
+      <c r="AO12" s="144"/>
+      <c r="AP12" s="146"/>
       <c r="AQ12" s="48" t="s">
         <v>122</v>
       </c>
@@ -9211,33 +9211,6 @@
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="AN11:AN12"/>
-    <mergeCell ref="AO11:AO12"/>
-    <mergeCell ref="AP11:AP12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="AJ11:AJ12"/>
-    <mergeCell ref="AM11:AM12"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="AJ9:AJ10"/>
-    <mergeCell ref="AM9:AM10"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="AJ6:AJ8"/>
-    <mergeCell ref="AM6:AM8"/>
-    <mergeCell ref="AJ2:AP2"/>
-    <mergeCell ref="V2:AB2"/>
-    <mergeCell ref="AC2:AI2"/>
-    <mergeCell ref="AN9:AN10"/>
-    <mergeCell ref="AO9:AO10"/>
-    <mergeCell ref="AP9:AP10"/>
-    <mergeCell ref="AN6:AN8"/>
-    <mergeCell ref="AO6:AO8"/>
-    <mergeCell ref="AP6:AP8"/>
     <mergeCell ref="B1:BQ1"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="C4:C5"/>
@@ -9254,6 +9227,33 @@
     <mergeCell ref="BI2:BQ2"/>
     <mergeCell ref="G2:U2"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="AJ2:AP2"/>
+    <mergeCell ref="V2:AB2"/>
+    <mergeCell ref="AC2:AI2"/>
+    <mergeCell ref="AN9:AN10"/>
+    <mergeCell ref="AO9:AO10"/>
+    <mergeCell ref="AP9:AP10"/>
+    <mergeCell ref="AN6:AN8"/>
+    <mergeCell ref="AO6:AO8"/>
+    <mergeCell ref="AP6:AP8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="AJ6:AJ8"/>
+    <mergeCell ref="AM6:AM8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="AJ9:AJ10"/>
+    <mergeCell ref="AM9:AM10"/>
+    <mergeCell ref="AN11:AN12"/>
+    <mergeCell ref="AO11:AO12"/>
+    <mergeCell ref="AP11:AP12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="AJ11:AJ12"/>
+    <mergeCell ref="AM11:AM12"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
@@ -9280,15 +9280,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005310FD7AD7CB004A8A6A0F373B4D2C9A" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e03df01192bc7a0d3daab74abc4d5196">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6400beab-f54b-4fe2-8a3b-8916a6012868" xmlns:ns3="af8b05c0-1ee2-463e-b79d-b3491b282b4f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c21e3be90755f8fba129abf768e1fac6" ns2:_="" ns3:_="">
     <xsd:import namespace="6400beab-f54b-4fe2-8a3b-8916a6012868"/>
@@ -9549,6 +9540,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{515C1B63-7175-4E1B-B42F-E31C07EF7985}">
   <ds:schemaRefs>
@@ -9567,14 +9567,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01D4BAD6-B1CF-44C3-8924-5E31C0B35D19}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9591,4 +9583,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA54D6B7-A2D4-4F0E-8A10-5B35BB83D50E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>